<commit_message>
Reporte ventas ML - 2026-04-11 21:00
</commit_message>
<xml_diff>
--- a/ventas_ml_historico.xlsx
+++ b/ventas_ml_historico.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI19"/>
+  <dimension ref="A1:AI37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -423,7 +423,7 @@
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="31" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="29" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
@@ -632,28 +632,28 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2000015920405788</v>
+        <v>2000015932875024</v>
       </c>
       <c r="B2" t="n">
-        <v>2000012446018577</v>
+        <v>2000012459011895</v>
       </c>
       <c r="C2" t="n">
-        <v>46825928963</v>
+        <v>46831837021</v>
       </c>
       <c r="D2" t="n">
-        <v>154112621330</v>
+        <v>153516147611</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>RODIBERTOROBLESALEJANDRO</t>
+          <t>LOAN2137132</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>2000015920405788</v>
+        <v>2000015932875024</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-04-10T07:55:11.000-04:00</t>
+          <t>2026-04-11T01:57:33.000-04:00</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -680,28 +680,28 @@
         <v>1</v>
       </c>
       <c r="M2" t="n">
-        <v>462</v>
+        <v>134.55</v>
       </c>
       <c r="N2" t="n">
-        <v>66.98999999999999</v>
+        <v>13.46</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>119.2</v>
+        <v>64</v>
       </c>
       <c r="Q2" t="n">
-        <v>59.6</v>
+        <v>32</v>
       </c>
       <c r="R2" t="n">
-        <v>59.6</v>
+        <v>32</v>
       </c>
       <c r="S2" t="n">
         <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>462</v>
+        <v>134.55</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
@@ -713,17 +713,17 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>75287834715773</t>
+          <t>75961294921402</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>MLM2381238905</t>
+          <t>MLM2541605311</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>Mercado Libre</t>
+          <t>Catálogo</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -733,16 +733,16 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>Bocina Power Bank Moreka 428 10w 5000mah Cables Tipo Ip Y C</t>
+          <t>Bocina Nebro Wg-131 Portátil Con Bluetooth Waterproof Azul</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="n">
-        <v>462</v>
+        <v>134.55</v>
       </c>
       <c r="AD2" t="inlineStr"/>
       <c r="AE2" t="n">
-        <v>293.59</v>
+        <v>76.91</v>
       </c>
       <c r="AF2" t="n">
         <v>0</v>
@@ -751,7 +751,7 @@
         <v>0</v>
       </c>
       <c r="AH2" t="n">
-        <v>66.98999999999999</v>
+        <v>13.46</v>
       </c>
       <c r="AI2" t="n">
         <v>0</v>
@@ -759,28 +759,26 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2000015919255616</v>
-      </c>
-      <c r="B3" t="n">
-        <v>2000012444792845</v>
-      </c>
+        <v>2000015932632586</v>
+      </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="n">
-        <v>46825583586</v>
+        <v>46831736271</v>
       </c>
       <c r="D3" t="n">
-        <v>153344481991</v>
+        <v>153514027567</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>MARTHACANDELARIALOPEZCORDOVA</t>
+          <t>ERVINEDUARDO RAMÍREZVZLA</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>2000015919255616</v>
+        <v>2000015932632586</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-04-10T02:48:35.000-04:00</t>
+          <t>2026-04-11T00:54:31.000-04:00</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -807,28 +805,28 @@
         <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>204.71</v>
+        <v>570.86</v>
       </c>
       <c r="N3" t="n">
-        <v>29.68</v>
+        <v>111.32</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="Q3" t="n">
-        <v>56</v>
+        <v>65.5</v>
       </c>
       <c r="R3" t="n">
-        <v>56</v>
+        <v>63.5</v>
       </c>
       <c r="S3" t="n">
         <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>204.71</v>
+        <v>570.86</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
@@ -840,12 +838,12 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>BR-KZNU-9NOO</t>
+          <t>74725206008902</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>MLM1904582897</t>
+          <t>MLM3712202158</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -860,16 +858,16 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>Bocina Moto Bluetooth Moreka W3s Tf Card Radio Fm Resistente</t>
+          <t>Cargador De Auto Moreka Cp0089 Starlink Mini Carga Rápida Negro</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr"/>
       <c r="AC3" t="n">
-        <v>204.71</v>
+        <v>570.86</v>
       </c>
       <c r="AD3" t="inlineStr"/>
       <c r="AE3" t="n">
-        <v>100.5</v>
+        <v>342.37</v>
       </c>
       <c r="AF3" t="n">
         <v>0</v>
@@ -878,7 +876,7 @@
         <v>0</v>
       </c>
       <c r="AH3" t="n">
-        <v>29.68</v>
+        <v>111.32</v>
       </c>
       <c r="AI3" t="n">
         <v>0</v>
@@ -886,26 +884,26 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2000015918864062</v>
+        <v>2000015932009672</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
-        <v>46825132377</v>
+        <v>46831746812</v>
       </c>
       <c r="D4" t="n">
-        <v>154084595658</v>
+        <v>153507878875</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ALEJANDRO3654</t>
+          <t>PLER973318</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>2000015918864062</v>
+        <v>2000015932009672</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-04-10T00:54:13.000-04:00</t>
+          <t>2026-04-10T23:10:48.000-04:00</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -932,28 +930,28 @@
         <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>198.75</v>
+        <v>429</v>
       </c>
       <c r="N4" t="n">
-        <v>28.82</v>
+        <v>62.2</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="Q4" t="n">
-        <v>34</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="R4" t="n">
-        <v>47</v>
+        <v>26.40000000000001</v>
       </c>
       <c r="S4" t="n">
         <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>198.75</v>
+        <v>429</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
@@ -965,12 +963,12 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>NN-TJ55-EIRE</t>
+          <t>76825709097220</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>MLM1904582897</t>
+          <t>MLM4762499328</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
@@ -985,16 +983,16 @@
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>Bocina Moto Bluetooth Moreka W3s Tf Card Radio Fm Resistente</t>
+          <t>Bocina Moreka A52 Bluetooth 15w Ipx6 1800mah</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="n">
-        <v>198.75</v>
+        <v>429</v>
       </c>
       <c r="AD4" t="inlineStr"/>
       <c r="AE4" t="n">
-        <v>117.94</v>
+        <v>260.36</v>
       </c>
       <c r="AF4" t="n">
         <v>0</v>
@@ -1003,7 +1001,7 @@
         <v>0</v>
       </c>
       <c r="AH4" t="n">
-        <v>28.82</v>
+        <v>62.2</v>
       </c>
       <c r="AI4" t="n">
         <v>0</v>
@@ -1011,28 +1009,28 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2000015918735504</v>
+        <v>2000015931967972</v>
       </c>
       <c r="B5" t="n">
-        <v>2000012444242337</v>
+        <v>2000012458078981</v>
       </c>
       <c r="C5" t="n">
-        <v>46825081431</v>
+        <v>46831734526</v>
       </c>
       <c r="D5" t="n">
-        <v>154083285822</v>
+        <v>154254282856</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>JLPACHECOS</t>
+          <t>HECTORPETITHECTORPETIT</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2000015918735504</v>
+        <v>2000015931967972</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-04-10T00:31:16.000-04:00</t>
+          <t>2026-04-10T23:07:11.000-04:00</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1059,28 +1057,28 @@
         <v>1</v>
       </c>
       <c r="M5" t="n">
-        <v>427.5</v>
+        <v>827.64</v>
       </c>
       <c r="N5" t="n">
-        <v>64.12</v>
+        <v>120.01</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>135.2</v>
+        <v>169</v>
       </c>
       <c r="Q5" t="n">
-        <v>67.59999999999999</v>
+        <v>84.5</v>
       </c>
       <c r="R5" t="n">
-        <v>67.59999999999999</v>
+        <v>84.5</v>
       </c>
       <c r="S5" t="n">
         <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>427.5</v>
+        <v>827.64</v>
       </c>
       <c r="U5" t="inlineStr">
         <is>
@@ -1092,12 +1090,12 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>A18/A38</t>
+          <t>76532580917858</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>MLM3442935972</t>
+          <t>MLM4545490694</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
@@ -1112,16 +1110,16 @@
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>10 Piezas De Micas Privacidad Cristal Templado 9d Oppo</t>
+          <t>Smart Watch Moreka R11 1.75  Ultra Hd Amoled Ipx68 Delgado</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="n">
-        <v>427.5</v>
+        <v>827.64</v>
       </c>
       <c r="AD5" t="inlineStr"/>
       <c r="AE5" t="n">
-        <v>257.09</v>
+        <v>548.21</v>
       </c>
       <c r="AF5" t="n">
         <v>0</v>
@@ -1130,7 +1128,7 @@
         <v>0</v>
       </c>
       <c r="AH5" t="n">
-        <v>64.12</v>
+        <v>120.01</v>
       </c>
       <c r="AI5" t="n">
         <v>0</v>
@@ -1138,28 +1136,28 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2000015918564930</v>
+        <v>2000015931930082</v>
       </c>
       <c r="B6" t="n">
-        <v>2000012444063601</v>
+        <v>2000012457998119</v>
       </c>
       <c r="C6" t="n">
-        <v>46825008245</v>
+        <v>46831420445</v>
       </c>
       <c r="D6" t="n">
-        <v>154081820206</v>
+        <v>154253338188</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>OSCARCOLOTL</t>
+          <t>CARLOSALFONZ</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2000015918564930</v>
+        <v>2000015931930082</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-04-10T00:03:34.000-04:00</t>
+          <t>2026-04-10T22:55:27.000-04:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1186,28 +1184,28 @@
         <v>1</v>
       </c>
       <c r="M6" t="n">
-        <v>164.45</v>
+        <v>3158.4</v>
       </c>
       <c r="N6" t="n">
-        <v>16.44</v>
+        <v>457.97</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>64</v>
+        <v>190</v>
       </c>
       <c r="Q6" t="n">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="R6" t="n">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="S6" t="n">
         <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>164.45</v>
+        <v>3158.4</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
@@ -1219,17 +1217,17 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>75961294921402</t>
+          <t>76867668365155</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>MLM2541605311</t>
+          <t>MLM4762499740</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>Catálogo</t>
+          <t>Mercado Libre</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
@@ -1239,16 +1237,16 @@
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>Bocina Nebro Wg-131 Portátil Con Bluetooth Waterproof Azul</t>
+          <t>Bocina Moreka A58 Bluetooth 230w Ipx6 2400mah</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="n">
-        <v>164.45</v>
+        <v>3158.4</v>
       </c>
       <c r="AD6" t="inlineStr"/>
       <c r="AE6" t="n">
-        <v>101.13</v>
+        <v>2319.54</v>
       </c>
       <c r="AF6" t="n">
         <v>0</v>
@@ -1257,7 +1255,7 @@
         <v>0</v>
       </c>
       <c r="AH6" t="n">
-        <v>16.44</v>
+        <v>457.97</v>
       </c>
       <c r="AI6" t="n">
         <v>0</v>
@@ -1265,28 +1263,28 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2000015915026216</v>
+        <v>2000015931187904</v>
       </c>
       <c r="B7" t="n">
-        <v>2000012440383505</v>
+        <v>2000012457258861</v>
       </c>
       <c r="C7" t="n">
-        <v>46823711622</v>
+        <v>46831390290</v>
       </c>
       <c r="D7" t="n">
-        <v>154052836286</v>
+        <v>154246400496</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>RAKE9550997</t>
+          <t>PEÑAHERNAN20221106222959</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2000015915026216</v>
+        <v>2000015931187904</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-04-09T19:18:46.000-04:00</t>
+          <t>2026-04-10T21:46:13.000-04:00</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1313,28 +1311,28 @@
         <v>1</v>
       </c>
       <c r="M7" t="n">
-        <v>234</v>
+        <v>925.3</v>
       </c>
       <c r="N7" t="n">
-        <v>23.4</v>
+        <v>92.53</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>275</v>
+        <v>190</v>
       </c>
       <c r="Q7" t="n">
-        <v>221</v>
+        <v>95</v>
       </c>
       <c r="R7" t="n">
-        <v>54</v>
+        <v>95</v>
       </c>
       <c r="S7" t="n">
         <v>0</v>
       </c>
       <c r="T7" t="n">
-        <v>234</v>
+        <v>925.3</v>
       </c>
       <c r="U7" t="inlineStr">
         <is>
@@ -1346,17 +1344,17 @@
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>75045745678283</t>
+          <t>BOCMORGRI+A18</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>MLM3813363284</t>
+          <t>MLM2335627661</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>Mercado Libre</t>
+          <t>Catálogo</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
@@ -1366,16 +1364,16 @@
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>Plug In 3.1a Usb Trasmisor Fm Bluetooth Carro Moreka Cp0073 Negro</t>
+          <t>Altavoz Bluetooth Moreka A18 70w Luces Led Ipx6 Portátil Radio Fm Tws Gris</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="n">
-        <v>234</v>
+        <v>925.3</v>
       </c>
       <c r="AD7" t="inlineStr"/>
       <c r="AE7" t="n">
-        <v>189.42</v>
+        <v>654.02</v>
       </c>
       <c r="AF7" t="n">
         <v>0</v>
@@ -1384,7 +1382,7 @@
         <v>0</v>
       </c>
       <c r="AH7" t="n">
-        <v>23.4</v>
+        <v>92.53</v>
       </c>
       <c r="AI7" t="n">
         <v>0</v>
@@ -1392,36 +1390,36 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2000015914539400</v>
+        <v>2000015930234104</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="n">
-        <v>46823497086</v>
+        <v>46830673091</v>
       </c>
       <c r="D8" t="n">
-        <v>153301992033</v>
+        <v>153488743041</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>VNUSROJIBLANK12</t>
+          <t>BOAL6432084</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>2000015914539400</v>
+        <v>2000015930234104</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-04-09T18:47:34.000-04:00</t>
+          <t>2026-04-10T20:22:43.000-04:00</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>paid</t>
+          <t>cancelled</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Pagado</t>
+          <t>Cancelado</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1438,28 +1436,28 @@
         <v>1</v>
       </c>
       <c r="M8" t="n">
-        <v>713</v>
+        <v>285</v>
       </c>
       <c r="N8" t="n">
-        <v>103.38</v>
+        <v>55.58</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>126</v>
+        <v>98</v>
       </c>
       <c r="Q8" t="n">
-        <v>84.5</v>
+        <v>39</v>
       </c>
       <c r="R8" t="n">
-        <v>41.5</v>
+        <v>59</v>
       </c>
       <c r="S8" t="n">
         <v>0</v>
       </c>
       <c r="T8" t="n">
-        <v>713</v>
+        <v>285</v>
       </c>
       <c r="U8" t="inlineStr">
         <is>
@@ -1471,12 +1469,12 @@
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>73239400752399</t>
+          <t>77343215226889</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>MLM3488485454</t>
+          <t>MLM5098643766</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
@@ -1491,16 +1489,16 @@
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>Smartwatch Pantalla Amoled 2600mah Resistente Al Agua</t>
+          <t>Combo Teclado Y Mouse Alámbrico Usb Español Laptop Ce-wd680 Gris</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="n">
-        <v>713</v>
+        <v>285</v>
       </c>
       <c r="AD8" t="inlineStr"/>
       <c r="AE8" t="n">
-        <v>460.58</v>
+        <v>164.62</v>
       </c>
       <c r="AF8" t="n">
         <v>0</v>
@@ -1509,7 +1507,7 @@
         <v>0</v>
       </c>
       <c r="AH8" t="n">
-        <v>103.38</v>
+        <v>55.58</v>
       </c>
       <c r="AI8" t="n">
         <v>0</v>
@@ -1517,28 +1515,28 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2000015914254952</v>
+        <v>2000015929551932</v>
       </c>
       <c r="B9" t="n">
-        <v>2000012439581533</v>
+        <v>2000012455537231</v>
       </c>
       <c r="C9" t="n">
-        <v>46823083335</v>
+        <v>46830373077</v>
       </c>
       <c r="D9" t="n">
-        <v>153298477411</v>
+        <v>153480488965</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>GA20240622001650</t>
+          <t>SOPORIESLAVERGAZONA817</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2000015914254952</v>
+        <v>2000015929551932</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-04-09T18:26:50.000-04:00</t>
+          <t>2026-04-10T19:30:38.000-04:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1562,31 +1560,31 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M9" t="n">
-        <v>322</v>
+        <v>795.24</v>
       </c>
       <c r="N9" t="n">
-        <v>31.4</v>
+        <v>115.31</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>160</v>
+        <v>445</v>
       </c>
       <c r="Q9" t="n">
-        <v>80</v>
+        <v>222.5</v>
       </c>
       <c r="R9" t="n">
-        <v>80</v>
+        <v>222.5</v>
       </c>
       <c r="S9" t="n">
         <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>322</v>
+        <v>795.24</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
@@ -1598,17 +1596,17 @@
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>72141399181305</t>
+          <t>76825905347021</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>MLM2289340133</t>
+          <t>MLM4762473244</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>Catálogo</t>
+          <t>Mercado Libre</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
@@ -1618,16 +1616,16 @@
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>Moreka K063 Power Bank Batería Portátil Carga Rápida 10000mah 4 Cables Púrpura</t>
+          <t>Bocina Moreka A50 Bluetooth 30w Ipx6 3600mah</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="n">
-        <v>161</v>
+        <v>795.24</v>
       </c>
       <c r="AD9" t="inlineStr"/>
       <c r="AE9" t="n">
-        <v>150.05</v>
+        <v>385.45</v>
       </c>
       <c r="AF9" t="n">
         <v>0</v>
@@ -1636,7 +1634,7 @@
         <v>0</v>
       </c>
       <c r="AH9" t="n">
-        <v>62.8</v>
+        <v>115.31</v>
       </c>
       <c r="AI9" t="n">
         <v>0</v>
@@ -1644,28 +1642,28 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2000015913353944</v>
+        <v>2000015929481304</v>
       </c>
       <c r="B10" t="n">
-        <v>2000012438644843</v>
+        <v>2000012455454135</v>
       </c>
       <c r="C10" t="n">
-        <v>46822944206</v>
+        <v>46830337829</v>
       </c>
       <c r="D10" t="n">
-        <v>153287496709</v>
+        <v>154225963480</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ESCI899332</t>
+          <t>VALERIAMARIASADAGARZA</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2000015913353944</v>
+        <v>2000015929481304</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-04-09T17:23:20.000-04:00</t>
+          <t>2026-04-10T19:24:38.000-04:00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1692,28 +1690,28 @@
         <v>1</v>
       </c>
       <c r="M10" t="n">
-        <v>164.45</v>
+        <v>237.5</v>
       </c>
       <c r="N10" t="n">
-        <v>16.44</v>
+        <v>42.75</v>
       </c>
       <c r="O10" t="n">
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>64</v>
+        <v>104.8</v>
       </c>
       <c r="Q10" t="n">
-        <v>32</v>
+        <v>52.4</v>
       </c>
       <c r="R10" t="n">
-        <v>32</v>
+        <v>52.4</v>
       </c>
       <c r="S10" t="n">
         <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>164.45</v>
+        <v>237.5</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
@@ -1725,17 +1723,17 @@
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>75961294921402</t>
+          <t>77490977902058</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>MLM2541605311</t>
+          <t>MLM2837538471</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>Catálogo</t>
+          <t>Mercado Libre</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
@@ -1745,16 +1743,16 @@
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>Bocina Nebro Wg-131 Portátil Con Bluetooth Waterproof Azul</t>
+          <t>Memoria Usb Kingston 16gb Data Traveler Se9 Metal Pendrive Blanca</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="n">
-        <v>164.45</v>
+        <v>237.5</v>
       </c>
       <c r="AD10" t="inlineStr"/>
       <c r="AE10" t="n">
-        <v>101.13</v>
+        <v>120.85</v>
       </c>
       <c r="AF10" t="n">
         <v>0</v>
@@ -1763,7 +1761,7 @@
         <v>0</v>
       </c>
       <c r="AH10" t="n">
-        <v>16.44</v>
+        <v>42.75</v>
       </c>
       <c r="AI10" t="n">
         <v>0</v>
@@ -1771,28 +1769,28 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2000015911947458</v>
+        <v>2000015927409710</v>
       </c>
       <c r="B11" t="n">
-        <v>2000012437174517</v>
+        <v>2000012453315257</v>
       </c>
       <c r="C11" t="n">
-        <v>46822254216</v>
+        <v>46829644948</v>
       </c>
       <c r="D11" t="n">
-        <v>154016435366</v>
+        <v>154195281014</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>MARAIDALIAAGUILERA</t>
+          <t>BIOTECVO</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2000015911947458</v>
+        <v>2000015927409710</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-04-09T15:43:23.000-04:00</t>
+          <t>2026-04-10T16:40:07.000-04:00</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1816,31 +1814,31 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M11" t="n">
-        <v>294.5</v>
+        <v>475</v>
       </c>
       <c r="N11" t="n">
-        <v>42.7</v>
+        <v>42.75</v>
       </c>
       <c r="O11" t="n">
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>152</v>
+        <v>209.6</v>
       </c>
       <c r="Q11" t="n">
-        <v>76</v>
+        <v>104.8</v>
       </c>
       <c r="R11" t="n">
-        <v>76</v>
+        <v>104.8</v>
       </c>
       <c r="S11" t="n">
         <v>0</v>
       </c>
       <c r="T11" t="n">
-        <v>294.5</v>
+        <v>475</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
@@ -1852,17 +1850,17 @@
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>AUDMORNEGM-921pack</t>
+          <t>77490977902058</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>MLM3356978052</t>
+          <t>MLM2837538471</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>Catálogo</t>
+          <t>Mercado Libre</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr">
@@ -1872,16 +1870,16 @@
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>Paquete 10 Audifonos Alámbricos Manos Libres Conector Tipo C Color Negro/blanco</t>
+          <t>Memoria Usb Kingston 16gb Data Traveler Se9 Metal Pendrive Blanca</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="n">
-        <v>294.5</v>
+        <v>237.5</v>
       </c>
       <c r="AD11" t="inlineStr"/>
       <c r="AE11" t="n">
-        <v>149.14</v>
+        <v>241.7</v>
       </c>
       <c r="AF11" t="n">
         <v>0</v>
@@ -1890,7 +1888,7 @@
         <v>0</v>
       </c>
       <c r="AH11" t="n">
-        <v>42.7</v>
+        <v>85.5</v>
       </c>
       <c r="AI11" t="n">
         <v>0</v>
@@ -1898,28 +1896,26 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>2000015911947456</v>
-      </c>
-      <c r="B12" t="n">
-        <v>2000012437174517</v>
-      </c>
+        <v>2000015926465502</v>
+      </c>
+      <c r="B12" t="inlineStr"/>
       <c r="C12" t="n">
-        <v>46822254216</v>
+        <v>46828912925</v>
       </c>
       <c r="D12" t="n">
-        <v>154016462860</v>
+        <v>154183216410</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>MARAIDALIAAGUILERA</t>
+          <t>JACOBOMIGUEL20230130120239</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2000015911947456</v>
+        <v>2000015926465502</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-04-09T15:43:23.000-04:00</t>
+          <t>2026-04-10T15:28:10.000-04:00</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1946,28 +1942,28 @@
         <v>1</v>
       </c>
       <c r="M12" t="n">
-        <v>294.5</v>
+        <v>109.8</v>
       </c>
       <c r="N12" t="n">
-        <v>42.7</v>
+        <v>13.18</v>
       </c>
       <c r="O12" t="n">
         <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>152</v>
+        <v>102</v>
       </c>
       <c r="Q12" t="n">
-        <v>76</v>
+        <v>40</v>
       </c>
       <c r="R12" t="n">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="S12" t="n">
         <v>0</v>
       </c>
       <c r="T12" t="n">
-        <v>294.5</v>
+        <v>109.8</v>
       </c>
       <c r="U12" t="inlineStr">
         <is>
@@ -1979,17 +1975,17 @@
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>76720994758426</t>
+          <t>SOPMORDEFMH-70B</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>MLM5115426106</t>
+          <t>MLM3357068774</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>Mercado Libre</t>
+          <t>Catálogo</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
@@ -1999,16 +1995,16 @@
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>Audífonos Moreka M-929 Alámbricos Manos Libres Jack 3.5mm Negro</t>
+          <t>Soporte De Celular Para Auto Estabilizador Para Motocicletas Color Default Title</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="n">
-        <v>294.5</v>
+        <v>109.8</v>
       </c>
       <c r="AD12" t="inlineStr"/>
       <c r="AE12" t="n">
-        <v>225.14</v>
+        <v>46.68</v>
       </c>
       <c r="AF12" t="n">
         <v>0</v>
@@ -2017,7 +2013,7 @@
         <v>0</v>
       </c>
       <c r="AH12" t="n">
-        <v>42.7</v>
+        <v>13.18</v>
       </c>
       <c r="AI12" t="n">
         <v>0</v>
@@ -2025,28 +2021,26 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2000015911035950</v>
-      </c>
-      <c r="B13" t="n">
-        <v>2000012436224727</v>
-      </c>
+        <v>2000015925898954</v>
+      </c>
+      <c r="B13" t="inlineStr"/>
       <c r="C13" t="n">
-        <v>46821806098</v>
+        <v>46828618943</v>
       </c>
       <c r="D13" t="n">
-        <v>154008453720</v>
+        <v>154176812930</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>HLALTAMIRANO</t>
+          <t>MEDINAVIANEY20220808095244</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2000015911035950</v>
+        <v>2000015925898954</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-04-09T14:44:05.000-04:00</t>
+          <t>2026-04-10T14:44:48.000-04:00</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -2073,28 +2067,28 @@
         <v>1</v>
       </c>
       <c r="M13" t="n">
-        <v>560.5</v>
+        <v>122</v>
       </c>
       <c r="N13" t="n">
-        <v>109.3</v>
+        <v>12.2</v>
       </c>
       <c r="O13" t="n">
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>131</v>
+        <v>89</v>
       </c>
       <c r="Q13" t="n">
-        <v>65.5</v>
+        <v>121</v>
       </c>
       <c r="R13" t="n">
-        <v>65.5</v>
+        <v>32</v>
       </c>
       <c r="S13" t="n">
         <v>0</v>
       </c>
       <c r="T13" t="n">
-        <v>560.5</v>
+        <v>122</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
@@ -2106,17 +2100,17 @@
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>74725206008902</t>
+          <t>76126320655919</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>MLM3712202158</t>
+          <t>MLM4676748386</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>Mercado Libre</t>
+          <t>Catálogo</t>
         </is>
       </c>
       <c r="Z13" t="inlineStr">
@@ -2126,16 +2120,16 @@
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>Cargador De Auto Moreka Cp0089 Starlink Mini Carga Rápida Negro</t>
+          <t>Audífonos In-ear Bluetooth 5.3 Moreka E601 Tws Blancos Con Estuche Carga Y Micrófono Blanco</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr"/>
       <c r="AC13" t="n">
-        <v>560.5</v>
+        <v>122</v>
       </c>
       <c r="AD13" t="inlineStr"/>
       <c r="AE13" t="n">
-        <v>334.96</v>
+        <v>0</v>
       </c>
       <c r="AF13" t="n">
         <v>0</v>
@@ -2144,7 +2138,7 @@
         <v>0</v>
       </c>
       <c r="AH13" t="n">
-        <v>109.3</v>
+        <v>0</v>
       </c>
       <c r="AI13" t="n">
         <v>0</v>
@@ -2152,26 +2146,28 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>2000015910487320</v>
-      </c>
-      <c r="B14" t="inlineStr"/>
+        <v>2000015925292404</v>
+      </c>
+      <c r="B14" t="n">
+        <v>2000012451099821</v>
+      </c>
       <c r="C14" t="n">
-        <v>46821271897</v>
+        <v>46828589732</v>
       </c>
       <c r="D14" t="n">
-        <v>153258785401</v>
+        <v>154170422818</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ENLACESS</t>
+          <t>VECE1241164</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2000015910487320</v>
+        <v>2000015925292404</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-04-09T14:10:04.000-04:00</t>
+          <t>2026-04-10T14:00:29.000-04:00</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -2198,28 +2194,28 @@
         <v>1</v>
       </c>
       <c r="M14" t="n">
-        <v>134.55</v>
+        <v>925.3</v>
       </c>
       <c r="N14" t="n">
-        <v>13.46</v>
+        <v>92.53</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>99</v>
+        <v>190</v>
       </c>
       <c r="Q14" t="n">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="R14" t="n">
-        <v>67</v>
+        <v>95</v>
       </c>
       <c r="S14" t="n">
         <v>0</v>
       </c>
       <c r="T14" t="n">
-        <v>134.55</v>
+        <v>925.3</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
@@ -2231,12 +2227,12 @@
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>75961290041531</t>
+          <t>BOCMORGRI+A18</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>MLM4318429096</t>
+          <t>MLM2335627661</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
@@ -2251,16 +2247,16 @@
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>Bocina Portátil Bluetooth Waterproof Mini Altavoz Inalámbric Negro</t>
+          <t>Altavoz Bluetooth Moreka A18 70w Luces Led Ipx6 Portátil Radio Fm Tws Gris</t>
         </is>
       </c>
       <c r="AB14" t="inlineStr"/>
       <c r="AC14" t="n">
-        <v>134.55</v>
+        <v>925.3</v>
       </c>
       <c r="AD14" t="inlineStr"/>
       <c r="AE14" t="n">
-        <v>76.91</v>
+        <v>654.02</v>
       </c>
       <c r="AF14" t="n">
         <v>0</v>
@@ -2269,7 +2265,7 @@
         <v>0</v>
       </c>
       <c r="AH14" t="n">
-        <v>13.46</v>
+        <v>92.53</v>
       </c>
       <c r="AI14" t="n">
         <v>0</v>
@@ -2277,28 +2273,28 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>2000015909133456</v>
+        <v>2000015924881136</v>
       </c>
       <c r="B15" t="n">
-        <v>2000012434212221</v>
+        <v>2000012450675355</v>
       </c>
       <c r="C15" t="n">
-        <v>46820912508</v>
+        <v>46828113793</v>
       </c>
       <c r="D15" t="n">
-        <v>153993729394</v>
+        <v>154166302560</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>ULY5205</t>
+          <t>BAÑUELOSJUAN20220718184511</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2000015909133456</v>
+        <v>2000015924881136</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-04-09T12:45:26.000-04:00</t>
+          <t>2026-04-10T13:31:12.000-04:00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2325,28 +2321,28 @@
         <v>1</v>
       </c>
       <c r="M15" t="n">
-        <v>189</v>
+        <v>228</v>
       </c>
       <c r="N15" t="n">
-        <v>31.18</v>
+        <v>22.8</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>64</v>
+        <v>285.52</v>
       </c>
       <c r="Q15" t="n">
-        <v>32</v>
+        <v>189.52</v>
       </c>
       <c r="R15" t="n">
-        <v>32</v>
+        <v>95.99999999999997</v>
       </c>
       <c r="S15" t="n">
         <v>0</v>
       </c>
       <c r="T15" t="n">
-        <v>189</v>
+        <v>228</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
@@ -2358,12 +2354,12 @@
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>BOCMORROK405</t>
+          <t>BOCMORROSMOR-410</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>MLM2972698110</t>
+          <t>MLM2883124554</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
@@ -2378,16 +2374,16 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>Bocina Para Moto Bluetooth Portátil 8w Resistente Al Agua</t>
+          <t>Mini Bocina Portátil Inalámbrico Bajo Tws Bluetooth Altavoz</t>
         </is>
       </c>
       <c r="AB15" t="inlineStr"/>
       <c r="AC15" t="n">
-        <v>189</v>
+        <v>228</v>
       </c>
       <c r="AD15" t="inlineStr"/>
       <c r="AE15" t="n">
-        <v>108.72</v>
+        <v>184.57</v>
       </c>
       <c r="AF15" t="n">
         <v>0</v>
@@ -2396,7 +2392,7 @@
         <v>0</v>
       </c>
       <c r="AH15" t="n">
-        <v>31.18</v>
+        <v>22.8</v>
       </c>
       <c r="AI15" t="n">
         <v>0</v>
@@ -2404,28 +2400,28 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>2000015901141806</v>
+        <v>2000015924881134</v>
       </c>
       <c r="B16" t="n">
-        <v>2000012425847369</v>
+        <v>2000012450675355</v>
       </c>
       <c r="C16" t="n">
-        <v>46816833391</v>
+        <v>46828113793</v>
       </c>
       <c r="D16" t="n">
-        <v>153164140863</v>
+        <v>153420099615</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>PC20241019154452</t>
+          <t>BAÑUELOSJUAN20220718184511</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2000015901141806</v>
+        <v>2000015924881134</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-04-08T21:27:21.000-04:00</t>
+          <t>2026-04-10T13:31:12.000-04:00</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2452,28 +2448,28 @@
         <v>1</v>
       </c>
       <c r="M16" t="n">
-        <v>167.9</v>
+        <v>228</v>
       </c>
       <c r="N16" t="n">
-        <v>25.18</v>
+        <v>22.8</v>
       </c>
       <c r="O16" t="n">
         <v>0</v>
       </c>
       <c r="P16" t="n">
-        <v>166</v>
+        <v>285.52</v>
       </c>
       <c r="Q16" t="n">
-        <v>134</v>
+        <v>189.52</v>
       </c>
       <c r="R16" t="n">
-        <v>32</v>
+        <v>95.99999999999997</v>
       </c>
       <c r="S16" t="n">
         <v>0</v>
       </c>
       <c r="T16" t="n">
-        <v>167.9</v>
+        <v>228</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
@@ -2485,12 +2481,12 @@
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>CARMORDEFP-203</t>
+          <t>BOCMORAZUMOR-410</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>MLM1912930539</t>
+          <t>MLM2883124554</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
@@ -2505,16 +2501,16 @@
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>Cargador Turbo Carga Rapida 20w Puerto Y Cable Tipo C P203 Blanco</t>
+          <t>Mini Bocina Portátil Inalámbrico Bajo Tws Bluetooth Altavoz</t>
         </is>
       </c>
       <c r="AB16" t="inlineStr"/>
       <c r="AC16" t="n">
-        <v>167.9</v>
+        <v>228</v>
       </c>
       <c r="AD16" t="inlineStr"/>
       <c r="AE16" t="n">
-        <v>18.7</v>
+        <v>184.57</v>
       </c>
       <c r="AF16" t="n">
         <v>0</v>
@@ -2523,7 +2519,7 @@
         <v>0</v>
       </c>
       <c r="AH16" t="n">
-        <v>0</v>
+        <v>22.8</v>
       </c>
       <c r="AI16" t="n">
         <v>0</v>
@@ -2531,28 +2527,26 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>2000015900479830</v>
-      </c>
-      <c r="B17" t="n">
-        <v>2000012425150469</v>
-      </c>
+        <v>2000015923571686</v>
+      </c>
+      <c r="B17" t="inlineStr"/>
       <c r="C17" t="n">
-        <v>46816813562</v>
+        <v>46827760364</v>
       </c>
       <c r="D17" t="n">
-        <v>153903764628</v>
+        <v>153405868355</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>GOJE20240421120542</t>
+          <t>VAZQUEZSARA20230812202049</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2000015900479830</v>
+        <v>2000015923571686</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-04-08T20:46:39.000-04:00</t>
+          <t>2026-04-10T11:59:16.000-04:00</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2579,28 +2573,28 @@
         <v>1</v>
       </c>
       <c r="M17" t="n">
-        <v>164.45</v>
+        <v>185</v>
       </c>
       <c r="N17" t="n">
-        <v>16.44</v>
+        <v>27.75</v>
       </c>
       <c r="O17" t="n">
         <v>0</v>
       </c>
       <c r="P17" t="n">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="Q17" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="R17" t="n">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="S17" t="n">
         <v>0</v>
       </c>
       <c r="T17" t="n">
-        <v>164.45</v>
+        <v>185</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
@@ -2612,12 +2606,12 @@
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>75961294921402</t>
+          <t>MULMORNEGmc-5848c</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>MLM2541605311</t>
+          <t>MLM3357041104</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
@@ -2632,16 +2626,16 @@
       </c>
       <c r="AA17" t="inlineStr">
         <is>
-          <t>Bocina Nebro Wg-131 Portátil Con Bluetooth Waterproof Azul</t>
+          <t>Multicontacto Moreka Mc-5848c 10 Tomas 1m Blanco 2 Usb Y Usb-c</t>
         </is>
       </c>
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="n">
-        <v>164.45</v>
+        <v>185</v>
       </c>
       <c r="AD17" t="inlineStr"/>
       <c r="AE17" t="n">
-        <v>101.13</v>
+        <v>102.5</v>
       </c>
       <c r="AF17" t="n">
         <v>0</v>
@@ -2650,7 +2644,7 @@
         <v>0</v>
       </c>
       <c r="AH17" t="n">
-        <v>16.44</v>
+        <v>27.75</v>
       </c>
       <c r="AI17" t="n">
         <v>0</v>
@@ -2658,28 +2652,28 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2000015898605836</v>
+        <v>2000015922863610</v>
       </c>
       <c r="B18" t="n">
-        <v>2000012423204427</v>
+        <v>2000012448562543</v>
       </c>
       <c r="C18" t="n">
-        <v>46815701425</v>
+        <v>46827137585</v>
       </c>
       <c r="D18" t="n">
-        <v>153887348360</v>
+        <v>153396288659</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>JG20241208202301</t>
+          <t>JORFERK</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2000015898605836</v>
+        <v>2000015922863610</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-04-08T18:56:03.000-04:00</t>
+          <t>2026-04-10T11:07:52.000-04:00</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2706,28 +2700,28 @@
         <v>1</v>
       </c>
       <c r="M18" t="n">
-        <v>164.45</v>
+        <v>713</v>
       </c>
       <c r="N18" t="n">
-        <v>16.44</v>
+        <v>103.38</v>
       </c>
       <c r="O18" t="n">
         <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>64</v>
+        <v>169</v>
       </c>
       <c r="Q18" t="n">
-        <v>32</v>
+        <v>84.5</v>
       </c>
       <c r="R18" t="n">
-        <v>32</v>
+        <v>84.5</v>
       </c>
       <c r="S18" t="n">
         <v>0</v>
       </c>
       <c r="T18" t="n">
-        <v>164.45</v>
+        <v>713</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
@@ -2739,17 +2733,17 @@
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>75961294921402</t>
+          <t>73239381698389</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>MLM2541605311</t>
+          <t>MLM3488449480</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>Catálogo</t>
+          <t>Mercado Libre</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr">
@@ -2759,16 +2753,16 @@
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>Bocina Nebro Wg-131 Portátil Con Bluetooth Waterproof Azul</t>
+          <t>Smartwatch Reloj Pantalla Amoled 330mah Resistente Al Agua</t>
         </is>
       </c>
       <c r="AB18" t="inlineStr"/>
       <c r="AC18" t="n">
-        <v>164.45</v>
+        <v>713</v>
       </c>
       <c r="AD18" t="inlineStr"/>
       <c r="AE18" t="n">
-        <v>101.13</v>
+        <v>460.58</v>
       </c>
       <c r="AF18" t="n">
         <v>0</v>
@@ -2777,7 +2771,7 @@
         <v>0</v>
       </c>
       <c r="AH18" t="n">
-        <v>16.44</v>
+        <v>103.38</v>
       </c>
       <c r="AI18" t="n">
         <v>0</v>
@@ -2785,28 +2779,28 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2000015897678942</v>
+        <v>2000015921193538</v>
       </c>
       <c r="B19" t="n">
-        <v>2000012422238933</v>
+        <v>2000012426900403</v>
       </c>
       <c r="C19" t="n">
-        <v>46815285151</v>
+        <v>46826592416</v>
       </c>
       <c r="D19" t="n">
-        <v>153133108857</v>
+        <v>153376320777</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>PIAD3222701</t>
+          <t>ALONDRAVIZUET</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2000015897678942</v>
+        <v>2000015921193538</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-04-08T17:58:14.000-04:00</t>
+          <t>2026-04-10T09:05:19.000-04:00</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2833,28 +2827,28 @@
         <v>1</v>
       </c>
       <c r="M19" t="n">
-        <v>840</v>
+        <v>954</v>
       </c>
       <c r="N19" t="n">
-        <v>121.8</v>
+        <v>138.33</v>
       </c>
       <c r="O19" t="n">
         <v>0</v>
       </c>
       <c r="P19" t="n">
-        <v>169</v>
+        <v>190</v>
       </c>
       <c r="Q19" t="n">
-        <v>84.5</v>
+        <v>95</v>
       </c>
       <c r="R19" t="n">
-        <v>84.5</v>
+        <v>95</v>
       </c>
       <c r="S19" t="n">
         <v>0</v>
       </c>
       <c r="T19" t="n">
-        <v>840</v>
+        <v>954</v>
       </c>
       <c r="U19" t="inlineStr">
         <is>
@@ -2866,12 +2860,12 @@
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>72368155667130</t>
+          <t>76825869750536</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>MLM2090316531</t>
+          <t>MLM4762485780</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
@@ -2886,27 +2880,2307 @@
       </c>
       <c r="AA19" t="inlineStr">
         <is>
-          <t>Paquete 20 Audifonos Alámbricos Manos Libres Conector Tipo C Negro/blanco</t>
+          <t>Bocina Moreka A48 Bluetooth 50w Ipx6 4000mah</t>
         </is>
       </c>
       <c r="AB19" t="inlineStr"/>
       <c r="AC19" t="n">
-        <v>840</v>
+        <v>954</v>
       </c>
       <c r="AD19" t="inlineStr"/>
       <c r="AE19" t="n">
+        <v>634.3200000000001</v>
+      </c>
+      <c r="AF19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH19" t="n">
+        <v>138.33</v>
+      </c>
+      <c r="AI19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2000015920405788</v>
+      </c>
+      <c r="B20" t="n">
+        <v>2000012446018577</v>
+      </c>
+      <c r="C20" t="n">
+        <v>46825928963</v>
+      </c>
+      <c r="D20" t="n">
+        <v>154112621330</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>RODIBERTOROBLESALEJANDRO</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>2000015920405788</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-04-10T07:55:11.000-04:00</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Pagado</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>1</v>
+      </c>
+      <c r="M20" t="n">
+        <v>462</v>
+      </c>
+      <c r="N20" t="n">
+        <v>66.98999999999999</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" t="n">
+        <v>119.2</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="R20" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="S20" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" t="n">
+        <v>462</v>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V20" t="n">
+        <v>0</v>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>75287834715773</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>MLM2381238905</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>Mercado Libre</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>Bocina Power Bank Moreka 428 10w 5000mah Cables Tipo Ip Y C</t>
+        </is>
+      </c>
+      <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="n">
+        <v>462</v>
+      </c>
+      <c r="AD20" t="inlineStr"/>
+      <c r="AE20" t="n">
+        <v>293.59</v>
+      </c>
+      <c r="AF20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH20" t="n">
+        <v>66.98999999999999</v>
+      </c>
+      <c r="AI20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>2000015919255616</v>
+      </c>
+      <c r="B21" t="n">
+        <v>2000012444792845</v>
+      </c>
+      <c r="C21" t="n">
+        <v>46825583586</v>
+      </c>
+      <c r="D21" t="n">
+        <v>153344481991</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>MARTHACANDELARIALOPEZCORDOVA</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>2000015919255616</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-04-10T02:48:35.000-04:00</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Pagado</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>1</v>
+      </c>
+      <c r="M21" t="n">
+        <v>204.71</v>
+      </c>
+      <c r="N21" t="n">
+        <v>29.68</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" t="n">
+        <v>112</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>56</v>
+      </c>
+      <c r="R21" t="n">
+        <v>56</v>
+      </c>
+      <c r="S21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T21" t="n">
+        <v>204.71</v>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V21" t="n">
+        <v>0</v>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>BR-KZNU-9NOO</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>MLM1904582897</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>Mercado Libre</t>
+        </is>
+      </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>Bocina Moto Bluetooth Moreka W3s Tf Card Radio Fm Resistente</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="n">
+        <v>204.71</v>
+      </c>
+      <c r="AD21" t="inlineStr"/>
+      <c r="AE21" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="AF21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH21" t="n">
+        <v>29.68</v>
+      </c>
+      <c r="AI21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>2000015918864062</v>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="n">
+        <v>46825132377</v>
+      </c>
+      <c r="D22" t="n">
+        <v>154084595658</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ALEJANDRO3654</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>2000015918864062</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-04-10T00:54:13.000-04:00</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Pagado</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L22" t="n">
+        <v>1</v>
+      </c>
+      <c r="M22" t="n">
+        <v>198.75</v>
+      </c>
+      <c r="N22" t="n">
+        <v>28.82</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" t="n">
+        <v>81</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>34</v>
+      </c>
+      <c r="R22" t="n">
+        <v>47</v>
+      </c>
+      <c r="S22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T22" t="n">
+        <v>198.75</v>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V22" t="n">
+        <v>0</v>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>NN-TJ55-EIRE</t>
+        </is>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>MLM1904582897</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>Mercado Libre</t>
+        </is>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>Bocina Moto Bluetooth Moreka W3s Tf Card Radio Fm Resistente</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="n">
+        <v>198.75</v>
+      </c>
+      <c r="AD22" t="inlineStr"/>
+      <c r="AE22" t="n">
+        <v>117.94</v>
+      </c>
+      <c r="AF22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH22" t="n">
+        <v>28.82</v>
+      </c>
+      <c r="AI22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>2000015918735504</v>
+      </c>
+      <c r="B23" t="n">
+        <v>2000012444242337</v>
+      </c>
+      <c r="C23" t="n">
+        <v>46825081431</v>
+      </c>
+      <c r="D23" t="n">
+        <v>154083285822</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>JLPACHECOS</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>2000015918735504</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-04-10T00:31:16.000-04:00</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Pagado</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L23" t="n">
+        <v>1</v>
+      </c>
+      <c r="M23" t="n">
+        <v>427.5</v>
+      </c>
+      <c r="N23" t="n">
+        <v>64.12</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" t="n">
+        <v>135.2</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="R23" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="S23" t="n">
+        <v>0</v>
+      </c>
+      <c r="T23" t="n">
+        <v>427.5</v>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V23" t="n">
+        <v>0</v>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>A18/A38</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>MLM3442935972</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>Mercado Libre</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>10 Piezas De Micas Privacidad Cristal Templado 9d Oppo</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="n">
+        <v>427.5</v>
+      </c>
+      <c r="AD23" t="inlineStr"/>
+      <c r="AE23" t="n">
+        <v>257.09</v>
+      </c>
+      <c r="AF23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH23" t="n">
+        <v>64.12</v>
+      </c>
+      <c r="AI23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>2000015918564930</v>
+      </c>
+      <c r="B24" t="n">
+        <v>2000012444063601</v>
+      </c>
+      <c r="C24" t="n">
+        <v>46825008245</v>
+      </c>
+      <c r="D24" t="n">
+        <v>154081820206</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>OSCARCOLOTL</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>2000015918564930</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2026-04-10T00:03:34.000-04:00</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Pagado</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
+        <v>1</v>
+      </c>
+      <c r="M24" t="n">
+        <v>164.45</v>
+      </c>
+      <c r="N24" t="n">
+        <v>16.44</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" t="n">
+        <v>64</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>32</v>
+      </c>
+      <c r="R24" t="n">
+        <v>32</v>
+      </c>
+      <c r="S24" t="n">
+        <v>0</v>
+      </c>
+      <c r="T24" t="n">
+        <v>164.45</v>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V24" t="n">
+        <v>0</v>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>75961294921402</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>MLM2541605311</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>Catálogo</t>
+        </is>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>Bocina Nebro Wg-131 Portátil Con Bluetooth Waterproof Azul</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="n">
+        <v>164.45</v>
+      </c>
+      <c r="AD24" t="inlineStr"/>
+      <c r="AE24" t="n">
+        <v>101.13</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH24" t="n">
+        <v>16.44</v>
+      </c>
+      <c r="AI24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>2000015915026216</v>
+      </c>
+      <c r="B25" t="n">
+        <v>2000012440383505</v>
+      </c>
+      <c r="C25" t="n">
+        <v>46823711622</v>
+      </c>
+      <c r="D25" t="n">
+        <v>154052836286</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>RAKE9550997</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>2000015915026216</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-04-09T19:18:46.000-04:00</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Pagado</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
+        <v>1</v>
+      </c>
+      <c r="M25" t="n">
+        <v>234</v>
+      </c>
+      <c r="N25" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" t="n">
+        <v>275</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>221</v>
+      </c>
+      <c r="R25" t="n">
+        <v>54</v>
+      </c>
+      <c r="S25" t="n">
+        <v>0</v>
+      </c>
+      <c r="T25" t="n">
+        <v>234</v>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V25" t="n">
+        <v>0</v>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>75045745678283</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>MLM3813363284</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>Mercado Libre</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>Plug In 3.1a Usb Trasmisor Fm Bluetooth Carro Moreka Cp0073 Negro</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="n">
+        <v>234</v>
+      </c>
+      <c r="AD25" t="inlineStr"/>
+      <c r="AE25" t="n">
+        <v>189.42</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH25" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="AI25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>2000015914539400</v>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="n">
+        <v>46823497086</v>
+      </c>
+      <c r="D26" t="n">
+        <v>153301992033</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>VNUSROJIBLANK12</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>2000015914539400</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-04-09T18:47:34.000-04:00</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Pagado</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L26" t="n">
+        <v>1</v>
+      </c>
+      <c r="M26" t="n">
+        <v>713</v>
+      </c>
+      <c r="N26" t="n">
+        <v>103.38</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" t="n">
+        <v>126</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="R26" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="S26" t="n">
+        <v>0</v>
+      </c>
+      <c r="T26" t="n">
+        <v>713</v>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V26" t="n">
+        <v>0</v>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>73239400752399</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>MLM3488485454</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>Mercado Libre</t>
+        </is>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>Smartwatch Pantalla Amoled 2600mah Resistente Al Agua</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr"/>
+      <c r="AC26" t="n">
+        <v>713</v>
+      </c>
+      <c r="AD26" t="inlineStr"/>
+      <c r="AE26" t="n">
+        <v>460.58</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH26" t="n">
+        <v>103.38</v>
+      </c>
+      <c r="AI26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>2000015914254952</v>
+      </c>
+      <c r="B27" t="n">
+        <v>2000012439581533</v>
+      </c>
+      <c r="C27" t="n">
+        <v>46823083335</v>
+      </c>
+      <c r="D27" t="n">
+        <v>153298477411</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>GA20240622001650</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>2000015914254952</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-04-09T18:26:50.000-04:00</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Pagado</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L27" t="n">
+        <v>2</v>
+      </c>
+      <c r="M27" t="n">
+        <v>322</v>
+      </c>
+      <c r="N27" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="n">
+        <v>160</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>80</v>
+      </c>
+      <c r="R27" t="n">
+        <v>80</v>
+      </c>
+      <c r="S27" t="n">
+        <v>0</v>
+      </c>
+      <c r="T27" t="n">
+        <v>322</v>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V27" t="n">
+        <v>0</v>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>72141399181305</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>MLM2289340133</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>Catálogo</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>Moreka K063 Power Bank Batería Portátil Carga Rápida 10000mah 4 Cables Púrpura</t>
+        </is>
+      </c>
+      <c r="AB27" t="inlineStr"/>
+      <c r="AC27" t="n">
+        <v>161</v>
+      </c>
+      <c r="AD27" t="inlineStr"/>
+      <c r="AE27" t="n">
+        <v>150.05</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH27" t="n">
+        <v>62.8</v>
+      </c>
+      <c r="AI27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>2000015913353944</v>
+      </c>
+      <c r="B28" t="n">
+        <v>2000012438644843</v>
+      </c>
+      <c r="C28" t="n">
+        <v>46822944206</v>
+      </c>
+      <c r="D28" t="n">
+        <v>153287496709</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>ESCI899332</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>2000015913353944</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2026-04-09T17:23:20.000-04:00</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Pagado</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L28" t="n">
+        <v>1</v>
+      </c>
+      <c r="M28" t="n">
+        <v>164.45</v>
+      </c>
+      <c r="N28" t="n">
+        <v>16.44</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" t="n">
+        <v>64</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>32</v>
+      </c>
+      <c r="R28" t="n">
+        <v>32</v>
+      </c>
+      <c r="S28" t="n">
+        <v>0</v>
+      </c>
+      <c r="T28" t="n">
+        <v>164.45</v>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V28" t="n">
+        <v>0</v>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>75961294921402</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>MLM2541605311</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>Catálogo</t>
+        </is>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>Bocina Nebro Wg-131 Portátil Con Bluetooth Waterproof Azul</t>
+        </is>
+      </c>
+      <c r="AB28" t="inlineStr"/>
+      <c r="AC28" t="n">
+        <v>164.45</v>
+      </c>
+      <c r="AD28" t="inlineStr"/>
+      <c r="AE28" t="n">
+        <v>101.13</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH28" t="n">
+        <v>16.44</v>
+      </c>
+      <c r="AI28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>2000015911947456</v>
+      </c>
+      <c r="B29" t="n">
+        <v>2000012437174517</v>
+      </c>
+      <c r="C29" t="n">
+        <v>46822254216</v>
+      </c>
+      <c r="D29" t="n">
+        <v>154016462860</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>MARAIDALIAAGUILERA</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>2000015911947456</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-04-09T15:43:23.000-04:00</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Pagado</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L29" t="n">
+        <v>1</v>
+      </c>
+      <c r="M29" t="n">
+        <v>294.5</v>
+      </c>
+      <c r="N29" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0</v>
+      </c>
+      <c r="P29" t="n">
+        <v>152</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>76</v>
+      </c>
+      <c r="R29" t="n">
+        <v>76</v>
+      </c>
+      <c r="S29" t="n">
+        <v>0</v>
+      </c>
+      <c r="T29" t="n">
+        <v>294.5</v>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V29" t="n">
+        <v>0</v>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>76720994758426</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>MLM5115426106</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>Mercado Libre</t>
+        </is>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>Audífonos Moreka M-929 Alámbricos Manos Libres Jack 3.5mm Negro</t>
+        </is>
+      </c>
+      <c r="AB29" t="inlineStr"/>
+      <c r="AC29" t="n">
+        <v>294.5</v>
+      </c>
+      <c r="AD29" t="inlineStr"/>
+      <c r="AE29" t="n">
+        <v>225.14</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH29" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="AI29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>2000015911947458</v>
+      </c>
+      <c r="B30" t="n">
+        <v>2000012437174517</v>
+      </c>
+      <c r="C30" t="n">
+        <v>46822254216</v>
+      </c>
+      <c r="D30" t="n">
+        <v>154016435366</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>MARAIDALIAAGUILERA</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>2000015911947458</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-04-09T15:43:23.000-04:00</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Pagado</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L30" t="n">
+        <v>1</v>
+      </c>
+      <c r="M30" t="n">
+        <v>294.5</v>
+      </c>
+      <c r="N30" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" t="n">
+        <v>152</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>76</v>
+      </c>
+      <c r="R30" t="n">
+        <v>76</v>
+      </c>
+      <c r="S30" t="n">
+        <v>0</v>
+      </c>
+      <c r="T30" t="n">
+        <v>294.5</v>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V30" t="n">
+        <v>0</v>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>AUDMORNEGM-921pack</t>
+        </is>
+      </c>
+      <c r="X30" t="inlineStr">
+        <is>
+          <t>MLM3356978052</t>
+        </is>
+      </c>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>Catálogo</t>
+        </is>
+      </c>
+      <c r="Z30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>Paquete 10 Audifonos Alámbricos Manos Libres Conector Tipo C Color Negro/blanco</t>
+        </is>
+      </c>
+      <c r="AB30" t="inlineStr"/>
+      <c r="AC30" t="n">
+        <v>294.5</v>
+      </c>
+      <c r="AD30" t="inlineStr"/>
+      <c r="AE30" t="n">
+        <v>149.14</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH30" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="AI30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>2000015911035950</v>
+      </c>
+      <c r="B31" t="n">
+        <v>2000012436224727</v>
+      </c>
+      <c r="C31" t="n">
+        <v>46821806098</v>
+      </c>
+      <c r="D31" t="n">
+        <v>154008453720</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>HLALTAMIRANO</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>2000015911035950</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-04-09T14:44:05.000-04:00</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Pagado</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L31" t="n">
+        <v>1</v>
+      </c>
+      <c r="M31" t="n">
+        <v>560.5</v>
+      </c>
+      <c r="N31" t="n">
+        <v>109.3</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" t="n">
+        <v>131</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="R31" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="S31" t="n">
+        <v>0</v>
+      </c>
+      <c r="T31" t="n">
+        <v>560.5</v>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V31" t="n">
+        <v>0</v>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>74725206008902</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>MLM3712202158</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>Mercado Libre</t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>Cargador De Auto Moreka Cp0089 Starlink Mini Carga Rápida Negro</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr"/>
+      <c r="AC31" t="n">
+        <v>560.5</v>
+      </c>
+      <c r="AD31" t="inlineStr"/>
+      <c r="AE31" t="n">
+        <v>334.96</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH31" t="n">
+        <v>109.3</v>
+      </c>
+      <c r="AI31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>2000015910487320</v>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="n">
+        <v>46821271897</v>
+      </c>
+      <c r="D32" t="n">
+        <v>153258785401</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>ENLACESS</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>2000015910487320</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-04-09T14:10:04.000-04:00</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Pagado</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L32" t="n">
+        <v>1</v>
+      </c>
+      <c r="M32" t="n">
+        <v>134.55</v>
+      </c>
+      <c r="N32" t="n">
+        <v>13.46</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" t="n">
+        <v>99</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>32</v>
+      </c>
+      <c r="R32" t="n">
+        <v>67</v>
+      </c>
+      <c r="S32" t="n">
+        <v>0</v>
+      </c>
+      <c r="T32" t="n">
+        <v>134.55</v>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V32" t="n">
+        <v>0</v>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>75961290041531</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>MLM4318429096</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>Catálogo</t>
+        </is>
+      </c>
+      <c r="Z32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>Bocina Portátil Bluetooth Waterproof Mini Altavoz Inalámbric Negro</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr"/>
+      <c r="AC32" t="n">
+        <v>134.55</v>
+      </c>
+      <c r="AD32" t="inlineStr"/>
+      <c r="AE32" t="n">
+        <v>76.91</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH32" t="n">
+        <v>13.46</v>
+      </c>
+      <c r="AI32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>2000015909133456</v>
+      </c>
+      <c r="B33" t="n">
+        <v>2000012434212221</v>
+      </c>
+      <c r="C33" t="n">
+        <v>46820912508</v>
+      </c>
+      <c r="D33" t="n">
+        <v>153993729394</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>ULY5205</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>2000015909133456</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-04-09T12:45:26.000-04:00</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Pagado</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L33" t="n">
+        <v>1</v>
+      </c>
+      <c r="M33" t="n">
+        <v>189</v>
+      </c>
+      <c r="N33" t="n">
+        <v>31.18</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0</v>
+      </c>
+      <c r="P33" t="n">
+        <v>64</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>32</v>
+      </c>
+      <c r="R33" t="n">
+        <v>32</v>
+      </c>
+      <c r="S33" t="n">
+        <v>0</v>
+      </c>
+      <c r="T33" t="n">
+        <v>189</v>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V33" t="n">
+        <v>0</v>
+      </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>BOCMORROK405</t>
+        </is>
+      </c>
+      <c r="X33" t="inlineStr">
+        <is>
+          <t>MLM2972698110</t>
+        </is>
+      </c>
+      <c r="Y33" t="inlineStr">
+        <is>
+          <t>Mercado Libre</t>
+        </is>
+      </c>
+      <c r="Z33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>Bocina Para Moto Bluetooth Portátil 8w Resistente Al Agua</t>
+        </is>
+      </c>
+      <c r="AB33" t="inlineStr"/>
+      <c r="AC33" t="n">
+        <v>189</v>
+      </c>
+      <c r="AD33" t="inlineStr"/>
+      <c r="AE33" t="n">
+        <v>108.72</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH33" t="n">
+        <v>31.18</v>
+      </c>
+      <c r="AI33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>2000015901141806</v>
+      </c>
+      <c r="B34" t="n">
+        <v>2000012425847369</v>
+      </c>
+      <c r="C34" t="n">
+        <v>46816833391</v>
+      </c>
+      <c r="D34" t="n">
+        <v>153164140863</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>PC20241019154452</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>2000015901141806</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-04-08T21:27:21.000-04:00</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Pagado</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L34" t="n">
+        <v>1</v>
+      </c>
+      <c r="M34" t="n">
+        <v>167.9</v>
+      </c>
+      <c r="N34" t="n">
+        <v>25.18</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" t="n">
+        <v>166</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>134</v>
+      </c>
+      <c r="R34" t="n">
+        <v>32</v>
+      </c>
+      <c r="S34" t="n">
+        <v>0</v>
+      </c>
+      <c r="T34" t="n">
+        <v>167.9</v>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V34" t="n">
+        <v>0</v>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>CARMORDEFP-203</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>MLM1912930539</t>
+        </is>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>Mercado Libre</t>
+        </is>
+      </c>
+      <c r="Z34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>Cargador Turbo Carga Rapida 20w Puerto Y Cable Tipo C P203 Blanco</t>
+        </is>
+      </c>
+      <c r="AB34" t="inlineStr"/>
+      <c r="AC34" t="n">
+        <v>167.9</v>
+      </c>
+      <c r="AD34" t="inlineStr"/>
+      <c r="AE34" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="AF34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>2000015900479830</v>
+      </c>
+      <c r="B35" t="n">
+        <v>2000012425150469</v>
+      </c>
+      <c r="C35" t="n">
+        <v>46816813562</v>
+      </c>
+      <c r="D35" t="n">
+        <v>153903764628</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>GOJE20240421120542</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>2000015900479830</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-04-08T20:46:39.000-04:00</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Pagado</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L35" t="n">
+        <v>1</v>
+      </c>
+      <c r="M35" t="n">
+        <v>164.45</v>
+      </c>
+      <c r="N35" t="n">
+        <v>16.44</v>
+      </c>
+      <c r="O35" t="n">
+        <v>0</v>
+      </c>
+      <c r="P35" t="n">
+        <v>64</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>32</v>
+      </c>
+      <c r="R35" t="n">
+        <v>32</v>
+      </c>
+      <c r="S35" t="n">
+        <v>0</v>
+      </c>
+      <c r="T35" t="n">
+        <v>164.45</v>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V35" t="n">
+        <v>0</v>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>75961294921402</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>MLM2541605311</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>Catálogo</t>
+        </is>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>Bocina Nebro Wg-131 Portátil Con Bluetooth Waterproof Azul</t>
+        </is>
+      </c>
+      <c r="AB35" t="inlineStr"/>
+      <c r="AC35" t="n">
+        <v>164.45</v>
+      </c>
+      <c r="AD35" t="inlineStr"/>
+      <c r="AE35" t="n">
+        <v>101.13</v>
+      </c>
+      <c r="AF35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH35" t="n">
+        <v>16.44</v>
+      </c>
+      <c r="AI35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>2000015898605836</v>
+      </c>
+      <c r="B36" t="n">
+        <v>2000012423204427</v>
+      </c>
+      <c r="C36" t="n">
+        <v>46815701425</v>
+      </c>
+      <c r="D36" t="n">
+        <v>153887348360</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>JG20241208202301</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>2000015898605836</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-04-08T18:56:03.000-04:00</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Pagado</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L36" t="n">
+        <v>1</v>
+      </c>
+      <c r="M36" t="n">
+        <v>164.45</v>
+      </c>
+      <c r="N36" t="n">
+        <v>16.44</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" t="n">
+        <v>64</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>32</v>
+      </c>
+      <c r="R36" t="n">
+        <v>32</v>
+      </c>
+      <c r="S36" t="n">
+        <v>0</v>
+      </c>
+      <c r="T36" t="n">
+        <v>164.45</v>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V36" t="n">
+        <v>0</v>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>75961294921402</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>MLM2541605311</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>Catálogo</t>
+        </is>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA36" t="inlineStr">
+        <is>
+          <t>Bocina Nebro Wg-131 Portátil Con Bluetooth Waterproof Azul</t>
+        </is>
+      </c>
+      <c r="AB36" t="inlineStr"/>
+      <c r="AC36" t="n">
+        <v>164.45</v>
+      </c>
+      <c r="AD36" t="inlineStr"/>
+      <c r="AE36" t="n">
+        <v>101.13</v>
+      </c>
+      <c r="AF36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH36" t="n">
+        <v>16.44</v>
+      </c>
+      <c r="AI36" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>2000015897678942</v>
+      </c>
+      <c r="B37" t="n">
+        <v>2000012422238933</v>
+      </c>
+      <c r="C37" t="n">
+        <v>46815285151</v>
+      </c>
+      <c r="D37" t="n">
+        <v>153133108857</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>PIAD3222701</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>2000015897678942</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-04-08T17:58:14.000-04:00</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Pagado</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L37" t="n">
+        <v>1</v>
+      </c>
+      <c r="M37" t="n">
+        <v>840</v>
+      </c>
+      <c r="N37" t="n">
+        <v>121.8</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" t="n">
+        <v>169</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="R37" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="S37" t="n">
+        <v>0</v>
+      </c>
+      <c r="T37" t="n">
+        <v>840</v>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V37" t="n">
+        <v>0</v>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>72368155667130</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>MLM2090316531</t>
+        </is>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>Mercado Libre</t>
+        </is>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AA37" t="inlineStr">
+        <is>
+          <t>Paquete 20 Audifonos Alámbricos Manos Libres Conector Tipo C Negro/blanco</t>
+        </is>
+      </c>
+      <c r="AB37" t="inlineStr"/>
+      <c r="AC37" t="n">
+        <v>840</v>
+      </c>
+      <c r="AD37" t="inlineStr"/>
+      <c r="AE37" t="n">
         <v>557.67</v>
       </c>
-      <c r="AF19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG19" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH19" t="n">
+      <c r="AF37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH37" t="n">
         <v>121.8</v>
       </c>
-      <c r="AI19" t="n">
+      <c r="AI37" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>